<commit_message>
Cập nhật thay thế Groq API bằng Ollama Cloud
</commit_message>
<xml_diff>
--- a/data/running_lists.xlsx
+++ b/data/running_lists.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="104">
   <si>
     <t>Link</t>
   </si>
@@ -276,6 +276,66 @@
   </si>
   <si>
     <t>phuluuhoang16081993@gmail.com</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/1167278443782686/</t>
+  </si>
+  <si>
+    <t>phuluuhoang168@gmail.com</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/541837446481848/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/809300869694777/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/189954891343066/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/vinfastgroupvietnam/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/739871613010588/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/SmartSolutionVinFast/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/2256706854847614/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/306267563852552/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/vinfastvfe34clubvn/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/vinfastvf5clubvnn/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/vinfastvf5clubvn/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/vf3vn/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/vinfastvf3clubvn/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/vf3clubvn369/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/1330938384935849/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/2824017314516168/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/3506649176245689/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/804472867906965/</t>
   </si>
 </sst>
 </file>
@@ -355,7 +415,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -363,7 +423,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -646,7 +705,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D75"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.26953125" bestFit="1" customWidth="1"/>
@@ -917,8 +976,8 @@
       <c r="C19" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="5">
-        <v>61577189999772</v>
+      <c r="D19" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -931,8 +990,8 @@
       <c r="C20" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="5">
-        <v>61577189999772</v>
+      <c r="D20" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -945,8 +1004,8 @@
       <c r="C21" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D21" s="5">
-        <v>61577189999772</v>
+      <c r="D21" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -959,8 +1018,8 @@
       <c r="C22" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="5">
-        <v>61577189999772</v>
+      <c r="D22" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -973,8 +1032,8 @@
       <c r="C23" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="5">
-        <v>61577189999772</v>
+      <c r="D23" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -987,8 +1046,8 @@
       <c r="C24" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="5">
-        <v>61577189999772</v>
+      <c r="D24" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -1001,8 +1060,8 @@
       <c r="C25" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="5">
-        <v>61577189999772</v>
+      <c r="D25" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -1015,8 +1074,8 @@
       <c r="C26" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="5">
-        <v>61577189999772</v>
+      <c r="D26" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -1029,8 +1088,8 @@
       <c r="C27" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="5">
-        <v>61577189999772</v>
+      <c r="D27" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
@@ -1043,8 +1102,8 @@
       <c r="C28" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D28" s="5">
-        <v>61577189999772</v>
+      <c r="D28" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -1057,8 +1116,8 @@
       <c r="C29" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D29" s="5">
-        <v>61577189999772</v>
+      <c r="D29" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
@@ -1071,8 +1130,8 @@
       <c r="C30" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D30" s="5">
-        <v>61577189999772</v>
+      <c r="D30" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
@@ -1085,8 +1144,8 @@
       <c r="C31" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D31" s="5">
-        <v>61577189999772</v>
+      <c r="D31" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
@@ -1099,8 +1158,8 @@
       <c r="C32" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D32" s="5">
-        <v>61577189999772</v>
+      <c r="D32" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -1113,8 +1172,8 @@
       <c r="C33" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D33" s="5">
-        <v>61577189999772</v>
+      <c r="D33" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
@@ -1127,8 +1186,8 @@
       <c r="C34" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D34" s="5">
-        <v>61577189999772</v>
+      <c r="D34" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -1141,8 +1200,8 @@
       <c r="C35" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D35" s="5">
-        <v>61577189999772</v>
+      <c r="D35" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -1155,8 +1214,8 @@
       <c r="C36" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D36" s="5">
-        <v>61577189999772</v>
+      <c r="D36" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
@@ -1169,8 +1228,8 @@
       <c r="C37" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D37" s="5">
-        <v>61577189999772</v>
+      <c r="D37" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -1183,8 +1242,8 @@
       <c r="C38" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D38" s="5">
-        <v>61577189999772</v>
+      <c r="D38" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -1620,7 +1679,382 @@
       <c r="D74" s="2"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C75" s="4"/>
+      <c r="A75" t="s">
+        <v>40</v>
+      </c>
+      <c r="B75" t="s">
+        <v>40</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>40</v>
+      </c>
+      <c r="B76" t="s">
+        <v>40</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>40</v>
+      </c>
+      <c r="B77" t="s">
+        <v>40</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>40</v>
+      </c>
+      <c r="B78" t="s">
+        <v>40</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>40</v>
+      </c>
+      <c r="B79" t="s">
+        <v>40</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>40</v>
+      </c>
+      <c r="B80" t="s">
+        <v>40</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>40</v>
+      </c>
+      <c r="B81" t="s">
+        <v>40</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>40</v>
+      </c>
+      <c r="B82" t="s">
+        <v>40</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>40</v>
+      </c>
+      <c r="B83" t="s">
+        <v>40</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>40</v>
+      </c>
+      <c r="B84" t="s">
+        <v>40</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>40</v>
+      </c>
+      <c r="B85" t="s">
+        <v>40</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>40</v>
+      </c>
+      <c r="B86" t="s">
+        <v>40</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>40</v>
+      </c>
+      <c r="B87" t="s">
+        <v>40</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>40</v>
+      </c>
+      <c r="B88" t="s">
+        <v>40</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>40</v>
+      </c>
+      <c r="B89" t="s">
+        <v>40</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>40</v>
+      </c>
+      <c r="B90" t="s">
+        <v>40</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>40</v>
+      </c>
+      <c r="B91" t="s">
+        <v>40</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>40</v>
+      </c>
+      <c r="B92" t="s">
+        <v>40</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>40</v>
+      </c>
+      <c r="B93" t="s">
+        <v>40</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>40</v>
+      </c>
+      <c r="B94" t="s">
+        <v>40</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D94" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>40</v>
+      </c>
+      <c r="B95" t="s">
+        <v>40</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>40</v>
+      </c>
+      <c r="B96" t="s">
+        <v>40</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>40</v>
+      </c>
+      <c r="B97" t="s">
+        <v>40</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>40</v>
+      </c>
+      <c r="B98" t="s">
+        <v>40</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>40</v>
+      </c>
+      <c r="B99" t="s">
+        <v>40</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>40</v>
+      </c>
+      <c r="B100" t="s">
+        <v>40</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>40</v>
+      </c>
+      <c r="B101" t="s">
+        <v>40</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>85</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1697,7 +2131,38 @@
     <hyperlink ref="C70" r:id="rId71"/>
     <hyperlink ref="C71" r:id="rId72"/>
     <hyperlink ref="C60" r:id="rId73"/>
+    <hyperlink ref="C75" r:id="rId74"/>
+    <hyperlink ref="D75" r:id="rId75"/>
+    <hyperlink ref="C76" r:id="rId76"/>
+    <hyperlink ref="C77" r:id="rId77"/>
+    <hyperlink ref="C78" r:id="rId78"/>
+    <hyperlink ref="C79" r:id="rId79"/>
+    <hyperlink ref="C80" r:id="rId80"/>
+    <hyperlink ref="C81" r:id="rId81"/>
+    <hyperlink ref="C82" r:id="rId82"/>
+    <hyperlink ref="C83" r:id="rId83"/>
+    <hyperlink ref="C84" r:id="rId84"/>
+    <hyperlink ref="C85" r:id="rId85"/>
+    <hyperlink ref="C86" r:id="rId86"/>
+    <hyperlink ref="C87" r:id="rId87"/>
+    <hyperlink ref="C88" r:id="rId88"/>
+    <hyperlink ref="C89" r:id="rId89"/>
+    <hyperlink ref="C90" r:id="rId90"/>
+    <hyperlink ref="C91" r:id="rId91"/>
+    <hyperlink ref="C92" r:id="rId92"/>
+    <hyperlink ref="C93" r:id="rId93"/>
+    <hyperlink ref="C94" r:id="rId94"/>
+    <hyperlink ref="C95" r:id="rId95"/>
+    <hyperlink ref="D76:D95" r:id="rId96" display="phuluuhoang168@gmail.com"/>
+    <hyperlink ref="C96" r:id="rId97"/>
+    <hyperlink ref="C97" r:id="rId98"/>
+    <hyperlink ref="C98" r:id="rId99"/>
+    <hyperlink ref="C99" r:id="rId100"/>
+    <hyperlink ref="C100" r:id="rId101"/>
+    <hyperlink ref="C101" r:id="rId102"/>
+    <hyperlink ref="D96:D101" r:id="rId103" display="phuluuhoang168@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId104"/>
 </worksheet>
 </file>
</xml_diff>